<commit_message>
add 2026 song videos to player, lyrics and song database
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/First of October Song Database.xlsx
+++ b/First of October Song Database.xlsx
@@ -8236,23 +8236,42 @@
       <c r="AF80" s="70" t="n"/>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="63">
-      <c r="A81" s="70" t="n"/>
-      <c r="B81" s="70" t="n"/>
-      <c r="C81" s="70" t="n"/>
-      <c r="D81" s="71" t="n"/>
-      <c r="E81" s="70" t="n"/>
-      <c r="F81" s="70" t="n"/>
-      <c r="G81" s="71" t="n"/>
-      <c r="H81" s="71" t="n"/>
-      <c r="I81" s="71" t="n"/>
-      <c r="J81" s="71" t="n"/>
-      <c r="K81" s="71" t="n"/>
-      <c r="L81" s="71" t="n"/>
-      <c r="M81" s="71" t="n"/>
-      <c r="N81" s="71" t="n"/>
-      <c r="O81" s="70" t="n"/>
-      <c r="P81" s="70" t="n"/>
-      <c r="Q81" s="70" t="n"/>
+      <c r="A81" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B81" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C81)</f>
+        <v/>
+      </c>
+      <c r="C81" s="84" t="inlineStr">
+        <is>
+          <t>ajlRK4GBU24</t>
+        </is>
+      </c>
+      <c r="D81" s="85" t="inlineStr">
+        <is>
+          <t>Thirtieth of September</t>
+        </is>
+      </c>
+      <c r="E81" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F81" s="86" t="n">
+        <v>0.04027777777777778</v>
+      </c>
+      <c r="G81" s="85" t="n"/>
+      <c r="H81" s="85" t="n"/>
+      <c r="I81" s="87" t="n"/>
+      <c r="J81" s="85" t="n"/>
+      <c r="K81" s="85" t="n"/>
+      <c r="L81" s="85" t="n"/>
+      <c r="M81" s="85" t="n"/>
+      <c r="N81" s="91" t="n"/>
+      <c r="O81" s="84" t="n"/>
+      <c r="P81" s="84" t="n"/>
+      <c r="Q81" s="84" t="n"/>
       <c r="R81" s="70" t="n"/>
       <c r="S81" s="70" t="n"/>
       <c r="T81" s="70" t="n"/>
@@ -8270,23 +8289,42 @@
       <c r="AF81" s="70" t="n"/>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="63">
-      <c r="A82" s="70" t="n"/>
-      <c r="B82" s="70" t="n"/>
-      <c r="C82" s="70" t="n"/>
-      <c r="D82" s="71" t="n"/>
-      <c r="E82" s="70" t="n"/>
-      <c r="F82" s="70" t="n"/>
-      <c r="G82" s="71" t="n"/>
-      <c r="H82" s="71" t="n"/>
-      <c r="I82" s="71" t="n"/>
-      <c r="J82" s="71" t="n"/>
-      <c r="K82" s="71" t="n"/>
-      <c r="L82" s="71" t="n"/>
-      <c r="M82" s="71" t="n"/>
-      <c r="N82" s="71" t="n"/>
-      <c r="O82" s="70" t="n"/>
-      <c r="P82" s="70" t="n"/>
-      <c r="Q82" s="70" t="n"/>
+      <c r="A82" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B82" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C82)</f>
+        <v/>
+      </c>
+      <c r="C82" s="84" t="inlineStr">
+        <is>
+          <t>a7A3NUMs6Hk</t>
+        </is>
+      </c>
+      <c r="D82" s="85" t="inlineStr">
+        <is>
+          <t>Sexy Ghost</t>
+        </is>
+      </c>
+      <c r="E82" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F82" s="86" t="n">
+        <v>0.1159722222222222</v>
+      </c>
+      <c r="G82" s="85" t="n"/>
+      <c r="H82" s="85" t="n"/>
+      <c r="I82" s="87" t="n"/>
+      <c r="J82" s="85" t="n"/>
+      <c r="K82" s="85" t="n"/>
+      <c r="L82" s="85" t="n"/>
+      <c r="M82" s="85" t="n"/>
+      <c r="N82" s="91" t="n"/>
+      <c r="O82" s="84" t="n"/>
+      <c r="P82" s="84" t="n"/>
+      <c r="Q82" s="84" t="n"/>
       <c r="R82" s="70" t="n"/>
       <c r="S82" s="70" t="n"/>
       <c r="T82" s="70" t="n"/>
@@ -8304,23 +8342,42 @@
       <c r="AF82" s="70" t="n"/>
     </row>
     <row r="83" ht="15.75" customHeight="1" s="63">
-      <c r="A83" s="70" t="n"/>
-      <c r="B83" s="70" t="n"/>
-      <c r="C83" s="70" t="n"/>
-      <c r="D83" s="71" t="n"/>
-      <c r="E83" s="70" t="n"/>
-      <c r="F83" s="70" t="n"/>
-      <c r="G83" s="71" t="n"/>
-      <c r="H83" s="71" t="n"/>
-      <c r="I83" s="71" t="n"/>
-      <c r="J83" s="71" t="n"/>
-      <c r="K83" s="71" t="n"/>
-      <c r="L83" s="71" t="n"/>
-      <c r="M83" s="71" t="n"/>
-      <c r="N83" s="71" t="n"/>
-      <c r="O83" s="70" t="n"/>
-      <c r="P83" s="70" t="n"/>
-      <c r="Q83" s="70" t="n"/>
+      <c r="A83" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B83" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C83)</f>
+        <v/>
+      </c>
+      <c r="C83" s="84" t="inlineStr">
+        <is>
+          <t>TgrshFRmO5c</t>
+        </is>
+      </c>
+      <c r="D83" s="85" t="inlineStr">
+        <is>
+          <t>Step Off My Grave</t>
+        </is>
+      </c>
+      <c r="E83" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F83" s="86" t="n">
+        <v>0.08611111111111111</v>
+      </c>
+      <c r="G83" s="85" t="n"/>
+      <c r="H83" s="85" t="n"/>
+      <c r="I83" s="87" t="n"/>
+      <c r="J83" s="85" t="n"/>
+      <c r="K83" s="85" t="n"/>
+      <c r="L83" s="85" t="n"/>
+      <c r="M83" s="85" t="n"/>
+      <c r="N83" s="91" t="n"/>
+      <c r="O83" s="84" t="n"/>
+      <c r="P83" s="84" t="n"/>
+      <c r="Q83" s="84" t="n"/>
       <c r="R83" s="70" t="n"/>
       <c r="S83" s="70" t="n"/>
       <c r="T83" s="70" t="n"/>
@@ -8338,23 +8395,42 @@
       <c r="AF83" s="70" t="n"/>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="63">
-      <c r="A84" s="70" t="n"/>
-      <c r="B84" s="70" t="n"/>
-      <c r="C84" s="70" t="n"/>
-      <c r="D84" s="71" t="n"/>
-      <c r="E84" s="70" t="n"/>
-      <c r="F84" s="70" t="n"/>
-      <c r="G84" s="71" t="n"/>
-      <c r="H84" s="71" t="n"/>
-      <c r="I84" s="71" t="n"/>
-      <c r="J84" s="71" t="n"/>
-      <c r="K84" s="71" t="n"/>
-      <c r="L84" s="71" t="n"/>
-      <c r="M84" s="71" t="n"/>
-      <c r="N84" s="71" t="n"/>
-      <c r="O84" s="70" t="n"/>
-      <c r="P84" s="70" t="n"/>
-      <c r="Q84" s="70" t="n"/>
+      <c r="A84" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B84" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C84)</f>
+        <v/>
+      </c>
+      <c r="C84" s="84" t="inlineStr">
+        <is>
+          <t>ejTZguANHW4</t>
+        </is>
+      </c>
+      <c r="D84" s="85" t="inlineStr">
+        <is>
+          <t>Apple Of My Eye</t>
+        </is>
+      </c>
+      <c r="E84" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F84" s="86" t="n">
+        <v>0.1305555555555556</v>
+      </c>
+      <c r="G84" s="85" t="n"/>
+      <c r="H84" s="85" t="n"/>
+      <c r="I84" s="87" t="n"/>
+      <c r="J84" s="85" t="n"/>
+      <c r="K84" s="85" t="n"/>
+      <c r="L84" s="85" t="n"/>
+      <c r="M84" s="85" t="n"/>
+      <c r="N84" s="91" t="n"/>
+      <c r="O84" s="84" t="n"/>
+      <c r="P84" s="84" t="n"/>
+      <c r="Q84" s="84" t="n"/>
       <c r="R84" s="70" t="n"/>
       <c r="S84" s="70" t="n"/>
       <c r="T84" s="70" t="n"/>
@@ -8372,23 +8448,42 @@
       <c r="AF84" s="70" t="n"/>
     </row>
     <row r="85" ht="15.75" customHeight="1" s="63">
-      <c r="A85" s="70" t="n"/>
-      <c r="B85" s="70" t="n"/>
-      <c r="C85" s="70" t="n"/>
-      <c r="D85" s="71" t="n"/>
-      <c r="E85" s="70" t="n"/>
-      <c r="F85" s="70" t="n"/>
-      <c r="G85" s="71" t="n"/>
-      <c r="H85" s="71" t="n"/>
-      <c r="I85" s="71" t="n"/>
-      <c r="J85" s="71" t="n"/>
-      <c r="K85" s="71" t="n"/>
-      <c r="L85" s="71" t="n"/>
-      <c r="M85" s="71" t="n"/>
-      <c r="N85" s="71" t="n"/>
-      <c r="O85" s="70" t="n"/>
-      <c r="P85" s="70" t="n"/>
-      <c r="Q85" s="70" t="n"/>
+      <c r="A85" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B85" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C85)</f>
+        <v/>
+      </c>
+      <c r="C85" s="84" t="inlineStr">
+        <is>
+          <t>Q2XJN5-HPEA</t>
+        </is>
+      </c>
+      <c r="D85" s="85" t="inlineStr">
+        <is>
+          <t>Here</t>
+        </is>
+      </c>
+      <c r="E85" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F85" s="86" t="n">
+        <v>0.19375</v>
+      </c>
+      <c r="G85" s="85" t="n"/>
+      <c r="H85" s="85" t="n"/>
+      <c r="I85" s="87" t="n"/>
+      <c r="J85" s="85" t="n"/>
+      <c r="K85" s="85" t="n"/>
+      <c r="L85" s="85" t="n"/>
+      <c r="M85" s="85" t="n"/>
+      <c r="N85" s="91" t="n"/>
+      <c r="O85" s="84" t="n"/>
+      <c r="P85" s="84" t="n"/>
+      <c r="Q85" s="84" t="n"/>
       <c r="R85" s="70" t="n"/>
       <c r="S85" s="70" t="n"/>
       <c r="T85" s="70" t="n"/>
@@ -8406,23 +8501,42 @@
       <c r="AF85" s="70" t="n"/>
     </row>
     <row r="86" ht="15.75" customHeight="1" s="63">
-      <c r="A86" s="70" t="n"/>
-      <c r="B86" s="70" t="n"/>
-      <c r="C86" s="70" t="n"/>
-      <c r="D86" s="71" t="n"/>
-      <c r="E86" s="70" t="n"/>
-      <c r="F86" s="70" t="n"/>
-      <c r="G86" s="71" t="n"/>
-      <c r="H86" s="71" t="n"/>
-      <c r="I86" s="71" t="n"/>
-      <c r="J86" s="71" t="n"/>
-      <c r="K86" s="71" t="n"/>
-      <c r="L86" s="71" t="n"/>
-      <c r="M86" s="71" t="n"/>
-      <c r="N86" s="71" t="n"/>
-      <c r="O86" s="70" t="n"/>
-      <c r="P86" s="70" t="n"/>
-      <c r="Q86" s="70" t="n"/>
+      <c r="A86" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B86" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C86)</f>
+        <v/>
+      </c>
+      <c r="C86" s="84" t="inlineStr">
+        <is>
+          <t>CJXHKWvZdvc</t>
+        </is>
+      </c>
+      <c r="D86" s="85" t="inlineStr">
+        <is>
+          <t>Fight With Dave Grohl</t>
+        </is>
+      </c>
+      <c r="E86" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F86" s="86" t="n">
+        <v>0.1069444444444444</v>
+      </c>
+      <c r="G86" s="85" t="n"/>
+      <c r="H86" s="85" t="n"/>
+      <c r="I86" s="87" t="n"/>
+      <c r="J86" s="85" t="n"/>
+      <c r="K86" s="85" t="n"/>
+      <c r="L86" s="85" t="n"/>
+      <c r="M86" s="85" t="n"/>
+      <c r="N86" s="91" t="n"/>
+      <c r="O86" s="84" t="n"/>
+      <c r="P86" s="84" t="n"/>
+      <c r="Q86" s="84" t="n"/>
       <c r="R86" s="70" t="n"/>
       <c r="S86" s="70" t="n"/>
       <c r="T86" s="70" t="n"/>
@@ -8440,23 +8554,42 @@
       <c r="AF86" s="70" t="n"/>
     </row>
     <row r="87" ht="15.75" customHeight="1" s="63">
-      <c r="A87" s="70" t="n"/>
-      <c r="B87" s="70" t="n"/>
-      <c r="C87" s="70" t="n"/>
-      <c r="D87" s="71" t="n"/>
-      <c r="E87" s="70" t="n"/>
-      <c r="F87" s="70" t="n"/>
-      <c r="G87" s="71" t="n"/>
-      <c r="H87" s="71" t="n"/>
-      <c r="I87" s="71" t="n"/>
-      <c r="J87" s="71" t="n"/>
-      <c r="K87" s="71" t="n"/>
-      <c r="L87" s="71" t="n"/>
-      <c r="M87" s="71" t="n"/>
-      <c r="N87" s="71" t="n"/>
-      <c r="O87" s="70" t="n"/>
-      <c r="P87" s="70" t="n"/>
-      <c r="Q87" s="70" t="n"/>
+      <c r="A87" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B87" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C87)</f>
+        <v/>
+      </c>
+      <c r="C87" s="84" t="inlineStr">
+        <is>
+          <t>uOy0oc9SJC4</t>
+        </is>
+      </c>
+      <c r="D87" s="85" t="inlineStr">
+        <is>
+          <t>Pick You Up, Take You Out</t>
+        </is>
+      </c>
+      <c r="E87" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F87" s="86" t="n">
+        <v>0.09236111111111112</v>
+      </c>
+      <c r="G87" s="85" t="n"/>
+      <c r="H87" s="85" t="n"/>
+      <c r="I87" s="87" t="n"/>
+      <c r="J87" s="85" t="n"/>
+      <c r="K87" s="85" t="n"/>
+      <c r="L87" s="85" t="n"/>
+      <c r="M87" s="85" t="n"/>
+      <c r="N87" s="91" t="n"/>
+      <c r="O87" s="84" t="n"/>
+      <c r="P87" s="84" t="n"/>
+      <c r="Q87" s="84" t="n"/>
       <c r="R87" s="70" t="n"/>
       <c r="S87" s="70" t="n"/>
       <c r="T87" s="70" t="n"/>
@@ -8474,23 +8607,42 @@
       <c r="AF87" s="70" t="n"/>
     </row>
     <row r="88" ht="15.75" customHeight="1" s="63">
-      <c r="A88" s="70" t="n"/>
-      <c r="B88" s="70" t="n"/>
-      <c r="C88" s="70" t="n"/>
-      <c r="D88" s="71" t="n"/>
-      <c r="E88" s="70" t="n"/>
-      <c r="F88" s="70" t="n"/>
-      <c r="G88" s="71" t="n"/>
-      <c r="H88" s="71" t="n"/>
-      <c r="I88" s="71" t="n"/>
-      <c r="J88" s="71" t="n"/>
-      <c r="K88" s="71" t="n"/>
-      <c r="L88" s="71" t="n"/>
-      <c r="M88" s="71" t="n"/>
-      <c r="N88" s="71" t="n"/>
-      <c r="O88" s="70" t="n"/>
-      <c r="P88" s="70" t="n"/>
-      <c r="Q88" s="70" t="n"/>
+      <c r="A88" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B88" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C88)</f>
+        <v/>
+      </c>
+      <c r="C88" s="84" t="inlineStr">
+        <is>
+          <t>Ovta5nDP7KE</t>
+        </is>
+      </c>
+      <c r="D88" s="85" t="inlineStr">
+        <is>
+          <t>Everyone Thinks That I'm Fine</t>
+        </is>
+      </c>
+      <c r="E88" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F88" s="86" t="n">
+        <v>0.03541666666666667</v>
+      </c>
+      <c r="G88" s="85" t="n"/>
+      <c r="H88" s="85" t="n"/>
+      <c r="I88" s="87" t="n"/>
+      <c r="J88" s="85" t="n"/>
+      <c r="K88" s="85" t="n"/>
+      <c r="L88" s="85" t="n"/>
+      <c r="M88" s="85" t="n"/>
+      <c r="N88" s="91" t="n"/>
+      <c r="O88" s="84" t="n"/>
+      <c r="P88" s="84" t="n"/>
+      <c r="Q88" s="84" t="n"/>
       <c r="R88" s="70" t="n"/>
       <c r="S88" s="70" t="n"/>
       <c r="T88" s="70" t="n"/>
@@ -8508,23 +8660,42 @@
       <c r="AF88" s="70" t="n"/>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="63">
-      <c r="A89" s="70" t="n"/>
-      <c r="B89" s="70" t="n"/>
-      <c r="C89" s="70" t="n"/>
-      <c r="D89" s="71" t="n"/>
-      <c r="E89" s="70" t="n"/>
-      <c r="F89" s="70" t="n"/>
-      <c r="G89" s="71" t="n"/>
-      <c r="H89" s="71" t="n"/>
-      <c r="I89" s="71" t="n"/>
-      <c r="J89" s="71" t="n"/>
-      <c r="K89" s="71" t="n"/>
-      <c r="L89" s="71" t="n"/>
-      <c r="M89" s="71" t="n"/>
-      <c r="N89" s="71" t="n"/>
-      <c r="O89" s="70" t="n"/>
-      <c r="P89" s="70" t="n"/>
-      <c r="Q89" s="70" t="n"/>
+      <c r="A89" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B89" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C89)</f>
+        <v/>
+      </c>
+      <c r="C89" s="84" t="inlineStr">
+        <is>
+          <t>j3Ss8LwjtDI</t>
+        </is>
+      </c>
+      <c r="D89" s="85" t="inlineStr">
+        <is>
+          <t>Rest Of My Life</t>
+        </is>
+      </c>
+      <c r="E89" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F89" s="86" t="n">
+        <v>0.10625</v>
+      </c>
+      <c r="G89" s="85" t="n"/>
+      <c r="H89" s="85" t="n"/>
+      <c r="I89" s="87" t="n"/>
+      <c r="J89" s="85" t="n"/>
+      <c r="K89" s="85" t="n"/>
+      <c r="L89" s="85" t="n"/>
+      <c r="M89" s="85" t="n"/>
+      <c r="N89" s="91" t="n"/>
+      <c r="O89" s="84" t="n"/>
+      <c r="P89" s="84" t="n"/>
+      <c r="Q89" s="84" t="n"/>
       <c r="R89" s="70" t="n"/>
       <c r="S89" s="70" t="n"/>
       <c r="T89" s="70" t="n"/>
@@ -8542,23 +8713,42 @@
       <c r="AF89" s="70" t="n"/>
     </row>
     <row r="90" ht="15.75" customHeight="1" s="63">
-      <c r="A90" s="70" t="n"/>
-      <c r="B90" s="70" t="n"/>
-      <c r="C90" s="70" t="n"/>
-      <c r="D90" s="71" t="n"/>
-      <c r="E90" s="70" t="n"/>
-      <c r="F90" s="70" t="n"/>
-      <c r="G90" s="71" t="n"/>
-      <c r="H90" s="71" t="n"/>
-      <c r="I90" s="71" t="n"/>
-      <c r="J90" s="71" t="n"/>
-      <c r="K90" s="71" t="n"/>
-      <c r="L90" s="71" t="n"/>
-      <c r="M90" s="71" t="n"/>
-      <c r="N90" s="71" t="n"/>
-      <c r="O90" s="70" t="n"/>
-      <c r="P90" s="70" t="n"/>
-      <c r="Q90" s="70" t="n"/>
+      <c r="A90" s="84" t="inlineStr">
+        <is>
+          <t>A Future Without You</t>
+        </is>
+      </c>
+      <c r="B90" s="67">
+        <f>_xlfn.CONCAT("https://youtube.com/watch/",C90)</f>
+        <v/>
+      </c>
+      <c r="C90" s="84" t="inlineStr">
+        <is>
+          <t>Hqm3Ivo93zY</t>
+        </is>
+      </c>
+      <c r="D90" s="85" t="inlineStr">
+        <is>
+          <t>I Can't Picture A Future Without You</t>
+        </is>
+      </c>
+      <c r="E90" s="84" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F90" s="86" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="G90" s="85" t="n"/>
+      <c r="H90" s="85" t="n"/>
+      <c r="I90" s="87" t="n"/>
+      <c r="J90" s="85" t="n"/>
+      <c r="K90" s="85" t="n"/>
+      <c r="L90" s="85" t="n"/>
+      <c r="M90" s="85" t="n"/>
+      <c r="N90" s="91" t="n"/>
+      <c r="O90" s="84" t="n"/>
+      <c r="P90" s="84" t="n"/>
+      <c r="Q90" s="84" t="n"/>
       <c r="R90" s="70" t="n"/>
       <c r="S90" s="70" t="n"/>
       <c r="T90" s="70" t="n"/>

</xml_diff>